<commit_message>
Accept Syncfusion 34.2.8 Word and Excel snapshots
</commit_message>
<xml_diff>
--- a/src/Tests/Samples.VerifyExcel.verified.xlsx
+++ b/src/Tests/Samples.VerifyExcel.verified.xlsx
@@ -107,7 +107,7 @@
     <t>Formula</t>
   </si>
   <si>
-    <t>https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzQuMS4yOQ==</t>
+    <t>https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzQuMi44</t>
   </si>
   <si>
     <r>
@@ -328,7 +328,7 @@
     <xdr:sp macro="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="0" name="TextBox 1">
-          <a:hlinkClick xmlns:p7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" p7:id="rId1" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzQuMS4yOQ=="/>
+          <a:hlinkClick xmlns:p7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" p7:id="rId1" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzQuMi44"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
@@ -2926,7 +2926,7 @@
     <mergeCell ref="A1001:T1001"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A1001" r:id="DeterministicId2" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzQuMS4yOQ==" display="Created with a trial version of Syncfusion Excel library or registered the wrong key in your application. Click here to obtain the valid key."/>
+    <hyperlink ref="A1001" r:id="DeterministicId2" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzQuMi44" display="Created with a trial version of Syncfusion Excel library or registered the wrong key in your application. Click here to obtain the valid key."/>
   </hyperlinks>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -2958,7 +2958,7 @@
     <mergeCell ref="A10:S10"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A10" r:id="DeterministicId1" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzQuMS4yOQ==" display="Created with a trial version of Syncfusion Excel library or registered the wrong key in your application. Click here to obtain the valid key."/>
+    <hyperlink ref="A10" r:id="DeterministicId1" tooltip="https://www.syncfusion.com/account/claim-license-key?pl=ZXhjZWwsc3ByZWFkc2hlZXRlZGl0b3IsZ3JpZHNkaw==&amp;vs=MzQuMi44" display="Created with a trial version of Syncfusion Excel library or registered the wrong key in your application. Click here to obtain the valid key."/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter scaleWithDoc="1" alignWithMargins="0" differentFirst="0" differentOddEven="0"/>

</xml_diff>

<commit_message>
Scrub OS locale from xlsx drawings; use DeterministicIoPackaging 1.0.0 protection scrubbing
Syncfusion stamps the text runs of drawings it adds (eg the trial watermark) with the
OS locale, not CurrentCulture, so xlsx snapshots differed between en-AU and en-US
machines. Replace the lang attribute with a fixed placeholder.

DeterministicIoPackaging 1.0.0 now scrubs password protection salt and hash, so drop
the local ScrubProtection.
</commit_message>
<xml_diff>
--- a/src/Tests/Samples.VerifyExcel.verified.xlsx
+++ b/src/Tests/Samples.VerifyExcel.verified.xlsx
@@ -353,7 +353,7 @@
         <a:bodyPr/>
         <a:p>
           <a:r>
-            <a:rPr lang="en-AU" b="1" i="0" sz="1200">
+            <a:rPr lang="DeterministicLang" b="1" i="0" sz="1200">
               <a:solidFill>
                 <a:srgbClr val="FF0000">
                   <a:alpha val="30000"/>
@@ -365,7 +365,7 @@
 wrong key in your application. Click</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-AU" b="1" i="0" sz="1200">
+            <a:rPr lang="DeterministicLang" b="1" i="0" sz="1200">
               <a:solidFill>
                 <a:srgbClr val="0563C1">
                   <a:alpha val="30000"/>
@@ -376,7 +376,7 @@
             <a:t> here</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-AU" b="1" i="0" sz="1200">
+            <a:rPr lang="DeterministicLang" b="1" i="0" sz="1200">
               <a:solidFill>
                 <a:srgbClr val="FF0000">
                   <a:alpha val="30000"/>
@@ -386,7 +386,7 @@
             </a:rPr>
             <a:t> to obtain the valid key.</a:t>
           </a:r>
-          <a:endParaRPr lang="en-AU" b="1" i="0" sz="1200">
+          <a:endParaRPr lang="DeterministicLang" b="1" i="0" sz="1200">
             <a:solidFill>
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
@@ -2953,7 +2953,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="DeterministicHash" saltValue="DeterministicSalt" spinCount="500" sheet="1" objects="1" scenarios="1" pivotTables="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA==" saltValue="AAAAAAAAAAAAAAAAAAAAAA==" spinCount="500" sheet="1" objects="1" scenarios="1" pivotTables="1"/>
   <mergeCells count="1">
     <mergeCell ref="A10:S10"/>
   </mergeCells>

</xml_diff>